<commit_message>
Refine invoice balance reconciliation and demo
</commit_message>
<xml_diff>
--- a/data/demo/demo_portfolio.xlsx
+++ b/data/demo/demo_portfolio.xlsx
@@ -160,7 +160,7 @@
     <tableColumn id="1" name="Invoice ID"/>
     <tableColumn id="2" name="Trade ID"/>
     <tableColumn id="3" name="Invoice Total"/>
-    <tableColumn id="4" name="Outstanding Amount"/>
+    <tableColumn id="4" name="Reported Outstanding Amount"/>
     <tableColumn id="5" name="Invoice Status"/>
     <tableColumn id="6" name="Notes"/>
   </tableColumns>
@@ -694,7 +694,7 @@
     <col width="12" customWidth="1" min="1" max="1"/>
     <col width="10" customWidth="1" min="2" max="2"/>
     <col width="15" customWidth="1" min="3" max="3"/>
-    <col width="20" customWidth="1" min="4" max="4"/>
+    <col width="29" customWidth="1" min="4" max="4"/>
     <col width="16" customWidth="1" min="5" max="5"/>
     <col width="40" customWidth="1" min="6" max="6"/>
   </cols>
@@ -717,7 +717,7 @@
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>Outstanding Amount</t>
+          <t>Reported Outstanding Amount</t>
         </is>
       </c>
       <c r="E1" t="inlineStr">

</xml_diff>